<commit_message>
adición de espectros del 25 y 29 de septiembre
</commit_message>
<xml_diff>
--- a/Datos ESPARTACO/Parámetros para análisis de Antares/Resultados absorción cobalto 2023.xlsx
+++ b/Datos ESPARTACO/Parámetros para análisis de Antares/Resultados absorción cobalto 2023.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -701,7 +701,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Octubre 12-2023</t>
+          <t>Septiembre 25-2023</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -715,36 +715,36 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>6563.884</v>
+        <v>6563.975</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>7.4e-05</t>
+          <t>8.8e-05</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>22.23</v>
+        <v>26.4</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.82</v>
+        <v>-1.06</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>0.54</v>
+        <v>0.55</v>
       </c>
       <c r="J7" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.93</v>
       </c>
       <c r="K7" t="n">
-        <v>0.6</v>
+        <v>0.59</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Octubre 19-2023</t>
+          <t>Septiembre 29-2023</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -758,18 +758,18 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>6563.888</v>
+        <v>6563.966</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>7.5e-05</t>
+          <t>8.7e-05</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>22.45</v>
+        <v>26</v>
       </c>
       <c r="G8" t="n">
-        <v>1.84</v>
+        <v>-0.58</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
@@ -778,9 +778,95 @@
         <v>0.55</v>
       </c>
       <c r="J8" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.59</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Octubre 12-2023</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Tierra</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Absorción Cobalto</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>6563.884</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>7.4e-05</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>22.23</v>
+      </c>
+      <c r="G9" t="n">
+        <v>-0.82</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Octubre 19-2023</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Tierra</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Absorción Cobalto</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>6563.888</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>7.5e-05</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>22.45</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="J10" t="n">
         <v>1.04</v>
       </c>
-      <c r="K8" t="n">
+      <c r="K10" t="n">
         <v>0.67</v>
       </c>
     </row>

</xml_diff>

<commit_message>
espectros 2023 completos c:
</commit_message>
<xml_diff>
--- a/Datos ESPARTACO/Parámetros para análisis de Antares/Resultados absorción cobalto 2023.xlsx
+++ b/Datos ESPARTACO/Parámetros para análisis de Antares/Resultados absorción cobalto 2023.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -701,7 +701,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Septiembre 25-2023</t>
+          <t>Septiembre 21-2023</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -715,18 +715,18 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>6563.975</v>
+        <v>6564.041</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.8e-05</t>
+          <t>9.8e-05</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>26.4</v>
+        <v>29.41</v>
       </c>
       <c r="G7" t="n">
-        <v>-1.06</v>
+        <v>1.24</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
@@ -735,16 +735,16 @@
         <v>0.55</v>
       </c>
       <c r="J7" t="n">
-        <v>0.93</v>
+        <v>0.97</v>
       </c>
       <c r="K7" t="n">
-        <v>0.59</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Septiembre 29-2023</t>
+          <t>Septiembre 25-2023</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -758,18 +758,18 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>6563.966</v>
+        <v>6563.975</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>8.7e-05</t>
+          <t>8.8e-05</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>26</v>
+        <v>26.4</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.58</v>
+        <v>-1.06</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
@@ -787,7 +787,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Octubre 12-2023</t>
+          <t>Septiembre 29-2023</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -801,36 +801,36 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>6563.884</v>
+        <v>6563.966</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>7.4e-05</t>
+          <t>8.7e-05</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>22.23</v>
+        <v>26</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.82</v>
+        <v>-0.58</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>0.54</v>
+        <v>0.55</v>
       </c>
       <c r="J9" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.93</v>
       </c>
       <c r="K9" t="n">
-        <v>0.6</v>
+        <v>0.59</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Octubre 19-2023</t>
+          <t>Octubre 12-2023</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -844,29 +844,72 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>6563.888</v>
+        <v>6563.884</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>7.5e-05</t>
+          <t>7.4e-05</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>22.45</v>
+        <v>22.23</v>
       </c>
       <c r="G10" t="n">
-        <v>1.84</v>
+        <v>-0.82</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
       </c>
       <c r="I10" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Octubre 19-2023</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Tierra</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Absorción Cobalto</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>6563.888</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>7.5e-05</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>22.45</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
         <v>0.55</v>
       </c>
-      <c r="J10" t="n">
+      <c r="J11" t="n">
         <v>1.04</v>
       </c>
-      <c r="K10" t="n">
+      <c r="K11" t="n">
         <v>0.67</v>
       </c>
     </row>

</xml_diff>